<commit_message>
fix: added modified xpath for cart button and updated testdata to match availabe products in the market
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Praveen\Coding Files\java\Flipkart-E2E-Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89163D20-331A-4BE8-94EA-530A3A7BFA89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4425B38B-C2E0-4452-A28C-654CD11264AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{C9B4D5A1-92A5-4738-9340-F2DB0B3CCAC9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C9B4D5A1-92A5-4738-9340-F2DB0B3CCAC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,16 +41,16 @@
     <t>Product name</t>
   </si>
   <si>
-    <t>Nothing phone 2a</t>
+    <t>Logitech g102</t>
   </si>
   <si>
-    <t>Nothing phone 3a</t>
+    <t>canon r100</t>
   </si>
   <si>
-    <t>Nikon D850</t>
+    <t>macbook neo</t>
   </si>
   <si>
-    <t>Logitech g102</t>
+    <t>nothing phone 3a</t>
   </si>
 </sst>
 </file>
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -122,7 +122,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2AB5945-4898-442E-9EC9-12A86FA614DE}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -465,44 +464,40 @@
     <col min="3" max="3" width="30.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="3"/>
     </row>
-    <row r="3" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="3"/>
     </row>
-    <row r="4" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: add allure dependencies to pom and update testrunner with allure report plugin
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Praveen\Coding Files\java\Flipkart-E2E-Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4425B38B-C2E0-4452-A28C-654CD11264AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BBA94F9-D5B0-4CC1-A3DF-DF8B9632DE7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C9B4D5A1-92A5-4738-9340-F2DB0B3CCAC9}"/>
+    <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="8880" xr2:uid="{C9B4D5A1-92A5-4738-9340-F2DB0B3CCAC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,9 +41,6 @@
     <t>Product name</t>
   </si>
   <si>
-    <t>Logitech g102</t>
-  </si>
-  <si>
     <t>canon r100</t>
   </si>
   <si>
@@ -51,6 +48,9 @@
   </si>
   <si>
     <t>nothing phone 3a</t>
+  </si>
+  <si>
+    <t>iphone 17</t>
   </si>
 </sst>
 </file>
@@ -473,28 +473,28 @@
     </row>
     <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
     <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
     </row>
     <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>

</xml_diff>